<commit_message>
update after final reviews
</commit_message>
<xml_diff>
--- a/manuscript/extended_data/ED_Table3_GeologicUnits.xlsx
+++ b/manuscript/extended_data/ED_Table3_GeologicUnits.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/phillipsm/Documents/Research/Publications/2025_Argyre_feldspar/manuscript/extended_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/phillipsm/Documents/Research/Publications/2025_Argyre_feldspar/manuscript/submission_materials/manuscript/extended_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58DF8F0E-9FB0-D94E-A6A1-0F56356EB808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1456D871-874F-5847-9E2A-DC55BA05CEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{72174BCA-D6B2-ED4D-B3CA-AC386D6366A1}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$6:$A$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$7:$A$15</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Argyre basin member 2'</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>(sic)</t>
+  </si>
+  <si>
+    <t>Geological Units from Dohm et al. 2015 used for uplifte material identification</t>
   </si>
 </sst>
 </file>
@@ -438,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2395F23E-CBF4-B84A-BBFD-8F8CFEC7856A}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.1640625" bestFit="1" customWidth="1"/>
@@ -447,13 +450,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
+      <c r="A1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -461,37 +464,42 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A8">
-    <sortCondition ref="A1:A8"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A9">
+    <sortCondition ref="A2:A9"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>